<commit_message>
feat: ra ov import
</commit_message>
<xml_diff>
--- a/samples/ra/2025 10 30 Royal Arch Visit Matrix 2025-26 Final Working Copy.xlsx
+++ b/samples/ra/2025 10 30 Royal Arch Visit Matrix 2025-26 Final Working Copy.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/kpturner/github/square_ov/samples/ra/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{821B488F-06A4-544B-896E-91E43724AC8A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{51ADB2A7-18AD-B84A-B26D-F68FF03E5DF6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="56140" yWindow="10160" windowWidth="29040" windowHeight="15720" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -150,7 +150,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1147" uniqueCount="337">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1148" uniqueCount="337">
   <si>
     <t xml:space="preserve"> </t>
   </si>
@@ -1482,7 +1482,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="6">
+  <borders count="7">
     <border>
       <left/>
       <right/>
@@ -1555,12 +1555,23 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="129">
+  <cellXfs count="130">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -1864,6 +1875,9 @@
       <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="19" fillId="0" borderId="0" xfId="1" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -8573,6 +8587,9 @@
       <c r="AX65" s="81"/>
     </row>
     <row r="66" spans="1:50" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A66" s="129" t="s">
+        <v>331</v>
+      </c>
       <c r="B66" t="s">
         <v>334</v>
       </c>

</xml_diff>

<commit_message>
feat: add rank order to the ai help
</commit_message>
<xml_diff>
--- a/samples/ra/2025 10 30 Royal Arch Visit Matrix 2025-26 Final Working Copy.xlsx
+++ b/samples/ra/2025 10 30 Royal Arch Visit Matrix 2025-26 Final Working Copy.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/kpturner/github/square_ov/samples/ra/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{51ADB2A7-18AD-B84A-B26D-F68FF03E5DF6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{58529FC1-8819-3740-865C-67DFEE703C90}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="56140" yWindow="10160" windowWidth="29040" windowHeight="15720" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2088,7 +2088,8 @@
     <col min="6" max="6" width="32.33203125" style="1" customWidth="1"/>
     <col min="7" max="7" width="15.83203125" customWidth="1"/>
     <col min="8" max="8" width="15.6640625" customWidth="1"/>
-    <col min="9" max="33" width="15.6640625" style="2" customWidth="1"/>
+    <col min="9" max="32" width="15.6640625" style="2" customWidth="1"/>
+    <col min="33" max="33" width="16.83203125" style="2" customWidth="1"/>
     <col min="34" max="35" width="15.6640625" style="2" hidden="1" customWidth="1"/>
     <col min="36" max="49" width="15.6640625" style="2" customWidth="1"/>
     <col min="50" max="50" width="14.6640625" style="2" customWidth="1"/>

</xml_diff>